<commit_message>
Ship SUGAR 1.4.0 QA and desktop workflow improvements
</commit_message>
<xml_diff>
--- a/examples/ghana-education-research/workspace/data/observations/ghana-demo-observations.xlsx
+++ b/examples/ghana-education-research/workspace/data/observations/ghana-demo-observations.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="observations" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'observations'!$A$1:$AP$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'observations'!$A$1:$AP$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP7"/>
+  <dimension ref="A1:AP6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -844,12 +844,12 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T21:45:48Z</t>
+          <t>2026-09-30T17:08:04Z</t>
         </is>
       </c>
       <c r="AO2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T21:45:48Z</t>
+          <t>2026-09-30T17:08:04Z</t>
         </is>
       </c>
       <c r="AP2" s="2" t="inlineStr">
@@ -1008,12 +1008,12 @@
       </c>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T21:45:48Z</t>
+          <t>2026-09-30T17:08:04Z</t>
         </is>
       </c>
       <c r="AO3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T21:45:48Z</t>
+          <t>2026-09-30T17:08:04Z</t>
         </is>
       </c>
       <c r="AP3" s="2" t="inlineStr">
@@ -1172,12 +1172,12 @@
       </c>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T21:45:48Z</t>
+          <t>2026-09-30T17:08:04Z</t>
         </is>
       </c>
       <c r="AO4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T21:45:48Z</t>
+          <t>2026-09-30T17:08:04Z</t>
         </is>
       </c>
       <c r="AP4" s="2" t="inlineStr">
@@ -1336,12 +1336,12 @@
       </c>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T21:45:48Z</t>
+          <t>2026-09-30T17:08:04Z</t>
         </is>
       </c>
       <c r="AO5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T21:45:48Z</t>
+          <t>2026-09-30T17:08:04Z</t>
         </is>
       </c>
       <c r="AP5" s="2" t="inlineStr">
@@ -1492,182 +1492,22 @@
       </c>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T21:45:48Z</t>
+          <t>2026-09-30T17:08:04Z</t>
         </is>
       </c>
       <c r="AO6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T21:45:48Z</t>
+          <t>2026-09-30T17:08:04Z</t>
         </is>
       </c>
       <c r="AP6" s="2" t="inlineStr">
-        <is>
-          <t>1.4</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>obs_aa332ec19c013ff2fd57</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>partnership</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>CIUG and Zhejiang University of Technology partnership</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>University of Ghana reports current CIUG board activity and work to strengthen its partnership with Zhejiang University of Technology.</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Confucius Institute at the University of Ghana, campus reference point</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Ghana</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="n">
-        <v>5.6465979</v>
-      </c>
-      <c r="L7" s="2" t="n">
-        <v>-0.188004</v>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>map_reference</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr"/>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>[{"basis": "map_reference", "city": "", "confidence": null, "country": "Ghana", "label": "Confucius Institute at the University of Ghana, campus reference point", "latitude": 5.6465979, "location_id": "loc_b837ca5bd7fb1ba85c51", "longitude": -0.188004, "note": "Campus reference point; not a building-level coordinate.", "precision": "locality", "region": "", "source_ref": "https://www.openstreetmap.org/way/308668766", "uncertainty_km": null}]</t>
-        </is>
-      </c>
-      <c r="P7" s="2" t="inlineStr">
-        <is>
-          <t>Confucius Institute at the University of Ghana</t>
-        </is>
-      </c>
-      <c r="Q7" s="2" t="inlineStr">
-        <is>
-          <t>Chinese language education and cultural programming</t>
-        </is>
-      </c>
-      <c r="R7" s="2" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="S7" s="2" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="T7" s="2" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U7" s="2" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V7" s="2" t="inlineStr"/>
-      <c r="W7" s="2" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X7" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="Y7" s="2" t="inlineStr"/>
-      <c r="Z7" s="2" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AA7" s="2" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AB7" s="2" t="inlineStr"/>
-      <c r="AC7" s="2" t="inlineStr"/>
-      <c r="AD7" s="2" t="inlineStr"/>
-      <c r="AE7" s="2" t="inlineStr"/>
-      <c r="AF7" s="2" t="inlineStr"/>
-      <c r="AG7" s="2" t="inlineStr">
-        <is>
-          <t>unreviewed</t>
-        </is>
-      </c>
-      <c r="AH7" s="2" t="inlineStr"/>
-      <c r="AI7" s="2" t="inlineStr"/>
-      <c r="AJ7" s="2" t="inlineStr">
-        <is>
-          <t>Public-source demo claim; analyst review is still required.</t>
-        </is>
-      </c>
-      <c r="AK7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.ug.edu.gh/news/ciug-board-meeting-charts-new-direction-2026-ug-and-zhejiang-university-technology-strengthen</t>
-        </is>
-      </c>
-      <c r="AL7" s="2" t="inlineStr">
-        <is>
-          <t>[{"archived_url": "", "collected_at": "2026-09-28T12:00:00Z", "language": "", "media_artifact_id": "", "media_locator": "", "native_id": "ciug-zjut-partnership", "note": "Paraphrased source record; inspect the linked source for the original wording.", "platform": "web", "published_at": "", "source_type": "official public webpage or document", "title": "CIUG and Zhejiang University of Technology partnership", "url": "https://www.ug.edu.gh/news/ciug-board-meeting-charts-new-direction-2026-ug-and-zhejiang-university-technology-strengthen"}]</t>
-        </is>
-      </c>
-      <c r="AM7" s="2" t="inlineStr">
-        <is>
-          <t>["web:ciug-zjut-partnership"]</t>
-        </is>
-      </c>
-      <c r="AN7" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28T21:45:48Z</t>
-        </is>
-      </c>
-      <c r="AO7" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28T21:45:48Z</t>
-        </is>
-      </c>
-      <c r="AP7" s="2" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AP7"/>
+  <autoFilter ref="A1:AP6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>